<commit_message>
etsy: orcamento TDAH sem cara de IA (ingles e frances, status em palavras, fotos novas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/adhd-budget/ADHD-Friendly-Budget.xlsx
+++ b/etsy/adhd-budget/ADHD-Friendly-Budget.xlsx
@@ -121,7 +121,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +130,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -144,12 +144,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4C2"/>
         <bgColor rgb="00FFF4C2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -193,16 +187,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
   </borders>
@@ -220,13 +214,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="13" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,11 +228,16 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -246,9 +245,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -262,13 +258,13 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -720,7 +716,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Money at a glance</t>
+          <t>Money overview</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -843,7 +839,7 @@
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>SUM(Bills!$C$6:$C$30)-SUMIFS(Bills!$C$6:$C$30,Bills!$E$6:$E$30,TRUE)</f>
+        <f>SUM(Bills!$C$6:$C$30)-SUMIFS(Bills!$C$6:$C$30,Bills!$E$6:$E$30,"Yes")</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -957,7 +953,7 @@
       </c>
       <c r="G13" s="1" t="n"/>
       <c r="H13" s="21">
-        <f>COUNTIFS(Bills!$F$6:$F$30,"Due in*")&amp;" bill(s) due in the next 3 days"</f>
+        <f>IF((COUNTIFS(Bills!$F$6:$F$30,"Due in*")+COUNTIFS(Bills!$F$6:$F$30,"Due today"))=0,"No bills due in the next 3 days",IF((COUNTIFS(Bills!$F$6:$F$30,"Due in*")+COUNTIFS(Bills!$F$6:$F$30,"Due today"))=1,"1 bill",(COUNTIFS(Bills!$F$6:$F$30,"Due in*")+COUNTIFS(Bills!$F$6:$F$30,"Due today"))&amp;" bills")&amp;" due in the next 3 days")</f>
         <v/>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -1012,7 +1008,7 @@
       </c>
       <c r="G15" s="1" t="n"/>
       <c r="H15" s="22">
-        <f>COUNTIFS(Bills!$F$6:$F$30,"⚠*")&amp;" bill(s) overdue"</f>
+        <f>IF(COUNTIFS(Bills!$F$6:$F$30,"Overdue")=0,"No overdue bills",IF(COUNTIFS(Bills!$F$6:$F$30,"Overdue")=1,"1 bill is overdue",COUNTIFS(Bills!$F$6:$F$30,"Overdue")&amp;" bills are overdue"))</f>
         <v/>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -1067,7 +1063,7 @@
       </c>
       <c r="G17" s="1" t="n"/>
       <c r="H17" s="23">
-        <f>COUNTIFS('Impulse List'!$E$6:$E$30,"⏳*")&amp;" item(s) cooling off on your Impulse List"</f>
+        <f>IF(COUNTIFS('Impulse List'!$E$6:$E$30,"Wait*")=0,"Nothing waiting on your Impulse List",IF(COUNTIFS('Impulse List'!$E$6:$E$30,"Wait*")=1,"1 item",COUNTIFS('Impulse List'!$E$6:$E$30,"Wait*")&amp;" items")&amp;" waiting on your Impulse List")</f>
         <v/>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -1829,6 +1825,21 @@
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>AND($C13&gt;0,$D13/$C13&gt;0.8,$D13/$C13&lt;=1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>LEFT(H13,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT(H15,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>LEFT(H17,7)="Nothing"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -1865,7 +1876,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start here: 3 steps, 5 minutes</t>
+          <t>Start here</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -1875,7 +1886,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only type in YELLOW cells. Everything else fills itself in.</t>
+          <t>Type only in the yellow cells. Everything else is calculated.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1916,7 +1927,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>Bills tab: list your bills once (amount + day of the month they are due).</t>
+          <t>Bills tab: list your bills once, with the amount and the day of the month they are due.</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -1936,7 +1947,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>Log tab: every time you spend or get paid, add ONE line: date, amount, category.</t>
+          <t>Log tab: each time you spend or get paid, add one line with the date, amount and category.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -1963,12 +1974,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>Dashboard: pick the month. The big number is what you can safely spend per day.</t>
+          <t>Dashboard: pick the month. The big number is what you can spend per day for the rest of it.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -1983,12 +1994,12 @@
       <c r="A15" s="1" t="n"/>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>Impulse List: want to buy something? Park it here for 48 hours first.</t>
+          <t>Impulse List: when you want to buy something, write it here and wait 48 hours.</t>
         </is>
       </c>
       <c r="D15" s="1" t="n"/>
@@ -2003,12 +2014,12 @@
       <c r="A17" s="1" t="n"/>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>🎯</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>Goals: watch your savings bars fill up.</t>
+          <t>Goals: update what you have saved and the bars fill up.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -2036,7 +2047,7 @@
       <c r="B21" s="1" t="n"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Tip: the example lines in Log, Bills and Goals are there to show how it works. Delete them and add yours.</t>
+          <t>The example lines in Log, Bills and Goals show how it works. Delete them and add your own.</t>
         </is>
       </c>
       <c r="D21" s="1" t="n"/>
@@ -2052,7 +2063,7 @@
       <c r="B23" s="1" t="n"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Works in Google Sheets (File → Import, or open the file in Drive) and in Microsoft Excel.</t>
+          <t>Works in Google Sheets (File &gt; Import, or open the file from Drive) and in Microsoft Excel.</t>
         </is>
       </c>
       <c r="D23" s="1" t="n"/>
@@ -3170,7 +3181,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Log: one line per money moment</t>
+          <t>Log: one line per purchase or payday</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -3183,7 +3194,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Date · Amount · Type · Category · Note. That's it.</t>
+          <t>Date, amount, type, category, and a note if you want.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -3471,7 +3482,7 @@
       </c>
       <c r="F15" s="27" t="inlineStr">
         <is>
-          <t>Shoes (was on the Impulse List!)</t>
+          <t>Shoes, from the Impulse List</t>
         </is>
       </c>
       <c r="G15" s="1" t="n"/>
@@ -4141,7 +4152,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Tick 'Paid' each month. Colours warn you before the due date.</t>
+          <t>Choose Yes under 'Paid?' each month. The colours warn you before the due date.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -4201,11 +4212,13 @@
       <c r="D6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="31" t="b">
-        <v>1</v>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F6" s="32">
-        <f>IF(B6="","",IF(E6=TRUE,"✓ Paid",IF(D6&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D6-DAY(TODAY())&lt;=3,"Due in "&amp;(D6-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D6))))</f>
+        <f>IF(B6="","",IF(E6="Yes","Paid",IF(D6&lt;DAY(TODAY()),"Overdue",IF((D6-DAY(TODAY()))=0,"Due today",IF((D6-DAY(TODAY()))&lt;=3,"Due in "&amp;(D6-DAY(TODAY()))&amp;IF((D6-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D6&amp;IF(AND(D6&gt;=11,D6&lt;=13),"th",IF(MOD(D6,10)=1,"st",IF(MOD(D6,10)=2,"nd",IF(MOD(D6,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G6" s="1" t="n"/>
@@ -4223,11 +4236,13 @@
       <c r="D7" s="30" t="n">
         <v>29</v>
       </c>
-      <c r="E7" s="31" t="b">
-        <v>0</v>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F7" s="32">
-        <f>IF(B7="","",IF(E7=TRUE,"✓ Paid",IF(D7&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D7-DAY(TODAY())&lt;=3,"Due in "&amp;(D7-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D7))))</f>
+        <f>IF(B7="","",IF(E7="Yes","Paid",IF(D7&lt;DAY(TODAY()),"Overdue",IF((D7-DAY(TODAY()))=0,"Due today",IF((D7-DAY(TODAY()))&lt;=3,"Due in "&amp;(D7-DAY(TODAY()))&amp;IF((D7-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D7&amp;IF(AND(D7&gt;=11,D7&lt;=13),"th",IF(MOD(D7,10)=1,"st",IF(MOD(D7,10)=2,"nd",IF(MOD(D7,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G7" s="1" t="n"/>
@@ -4245,11 +4260,13 @@
       <c r="D8" s="30" t="n">
         <v>15</v>
       </c>
-      <c r="E8" s="31" t="b">
-        <v>1</v>
+      <c r="E8" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F8" s="32">
-        <f>IF(B8="","",IF(E8=TRUE,"✓ Paid",IF(D8&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D8-DAY(TODAY())&lt;=3,"Due in "&amp;(D8-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D8))))</f>
+        <f>IF(B8="","",IF(E8="Yes","Paid",IF(D8&lt;DAY(TODAY()),"Overdue",IF((D8-DAY(TODAY()))=0,"Due today",IF((D8-DAY(TODAY()))&lt;=3,"Due in "&amp;(D8-DAY(TODAY()))&amp;IF((D8-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D8&amp;IF(AND(D8&gt;=11,D8&lt;=13),"th",IF(MOD(D8,10)=1,"st",IF(MOD(D8,10)=2,"nd",IF(MOD(D8,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G8" s="1" t="n"/>
@@ -4267,11 +4284,13 @@
       <c r="D9" s="30" t="n">
         <v>30</v>
       </c>
-      <c r="E9" s="31" t="b">
-        <v>0</v>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F9" s="32">
-        <f>IF(B9="","",IF(E9=TRUE,"✓ Paid",IF(D9&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D9-DAY(TODAY())&lt;=3,"Due in "&amp;(D9-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D9))))</f>
+        <f>IF(B9="","",IF(E9="Yes","Paid",IF(D9&lt;DAY(TODAY()),"Overdue",IF((D9-DAY(TODAY()))=0,"Due today",IF((D9-DAY(TODAY()))&lt;=3,"Due in "&amp;(D9-DAY(TODAY()))&amp;IF((D9-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D9&amp;IF(AND(D9&gt;=11,D9&lt;=13),"th",IF(MOD(D9,10)=1,"st",IF(MOD(D9,10)=2,"nd",IF(MOD(D9,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G9" s="1" t="n"/>
@@ -4289,11 +4308,13 @@
       <c r="D10" s="30" t="n">
         <v>24</v>
       </c>
-      <c r="E10" s="31" t="b">
-        <v>0</v>
+      <c r="E10" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F10" s="32">
-        <f>IF(B10="","",IF(E10=TRUE,"✓ Paid",IF(D10&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D10-DAY(TODAY())&lt;=3,"Due in "&amp;(D10-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D10))))</f>
+        <f>IF(B10="","",IF(E10="Yes","Paid",IF(D10&lt;DAY(TODAY()),"Overdue",IF((D10-DAY(TODAY()))=0,"Due today",IF((D10-DAY(TODAY()))&lt;=3,"Due in "&amp;(D10-DAY(TODAY()))&amp;IF((D10-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D10&amp;IF(AND(D10&gt;=11,D10&lt;=13),"th",IF(MOD(D10,10)=1,"st",IF(MOD(D10,10)=2,"nd",IF(MOD(D10,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G10" s="1" t="n"/>
@@ -4311,11 +4332,13 @@
       <c r="D11" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="31" t="b">
-        <v>1</v>
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F11" s="32">
-        <f>IF(B11="","",IF(E11=TRUE,"✓ Paid",IF(D11&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D11-DAY(TODAY())&lt;=3,"Due in "&amp;(D11-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D11))))</f>
+        <f>IF(B11="","",IF(E11="Yes","Paid",IF(D11&lt;DAY(TODAY()),"Overdue",IF((D11-DAY(TODAY()))=0,"Due today",IF((D11-DAY(TODAY()))&lt;=3,"Due in "&amp;(D11-DAY(TODAY()))&amp;IF((D11-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D11&amp;IF(AND(D11&gt;=11,D11&lt;=13),"th",IF(MOD(D11,10)=1,"st",IF(MOD(D11,10)=2,"nd",IF(MOD(D11,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G11" s="1" t="n"/>
@@ -4327,7 +4350,7 @@
       <c r="D12" s="30" t="n"/>
       <c r="E12" s="31" t="n"/>
       <c r="F12" s="32">
-        <f>IF(B12="","",IF(E12=TRUE,"✓ Paid",IF(D12&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D12-DAY(TODAY())&lt;=3,"Due in "&amp;(D12-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D12))))</f>
+        <f>IF(B12="","",IF(E12="Yes","Paid",IF(D12&lt;DAY(TODAY()),"Overdue",IF((D12-DAY(TODAY()))=0,"Due today",IF((D12-DAY(TODAY()))&lt;=3,"Due in "&amp;(D12-DAY(TODAY()))&amp;IF((D12-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D12&amp;IF(AND(D12&gt;=11,D12&lt;=13),"th",IF(MOD(D12,10)=1,"st",IF(MOD(D12,10)=2,"nd",IF(MOD(D12,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G12" s="1" t="n"/>
@@ -4339,7 +4362,7 @@
       <c r="D13" s="30" t="n"/>
       <c r="E13" s="31" t="n"/>
       <c r="F13" s="32">
-        <f>IF(B13="","",IF(E13=TRUE,"✓ Paid",IF(D13&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D13-DAY(TODAY())&lt;=3,"Due in "&amp;(D13-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D13))))</f>
+        <f>IF(B13="","",IF(E13="Yes","Paid",IF(D13&lt;DAY(TODAY()),"Overdue",IF((D13-DAY(TODAY()))=0,"Due today",IF((D13-DAY(TODAY()))&lt;=3,"Due in "&amp;(D13-DAY(TODAY()))&amp;IF((D13-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D13&amp;IF(AND(D13&gt;=11,D13&lt;=13),"th",IF(MOD(D13,10)=1,"st",IF(MOD(D13,10)=2,"nd",IF(MOD(D13,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G13" s="1" t="n"/>
@@ -4351,7 +4374,7 @@
       <c r="D14" s="30" t="n"/>
       <c r="E14" s="31" t="n"/>
       <c r="F14" s="32">
-        <f>IF(B14="","",IF(E14=TRUE,"✓ Paid",IF(D14&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D14-DAY(TODAY())&lt;=3,"Due in "&amp;(D14-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D14))))</f>
+        <f>IF(B14="","",IF(E14="Yes","Paid",IF(D14&lt;DAY(TODAY()),"Overdue",IF((D14-DAY(TODAY()))=0,"Due today",IF((D14-DAY(TODAY()))&lt;=3,"Due in "&amp;(D14-DAY(TODAY()))&amp;IF((D14-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D14&amp;IF(AND(D14&gt;=11,D14&lt;=13),"th",IF(MOD(D14,10)=1,"st",IF(MOD(D14,10)=2,"nd",IF(MOD(D14,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G14" s="1" t="n"/>
@@ -4363,7 +4386,7 @@
       <c r="D15" s="30" t="n"/>
       <c r="E15" s="31" t="n"/>
       <c r="F15" s="32">
-        <f>IF(B15="","",IF(E15=TRUE,"✓ Paid",IF(D15&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D15-DAY(TODAY())&lt;=3,"Due in "&amp;(D15-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D15))))</f>
+        <f>IF(B15="","",IF(E15="Yes","Paid",IF(D15&lt;DAY(TODAY()),"Overdue",IF((D15-DAY(TODAY()))=0,"Due today",IF((D15-DAY(TODAY()))&lt;=3,"Due in "&amp;(D15-DAY(TODAY()))&amp;IF((D15-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D15&amp;IF(AND(D15&gt;=11,D15&lt;=13),"th",IF(MOD(D15,10)=1,"st",IF(MOD(D15,10)=2,"nd",IF(MOD(D15,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G15" s="1" t="n"/>
@@ -4375,7 +4398,7 @@
       <c r="D16" s="30" t="n"/>
       <c r="E16" s="31" t="n"/>
       <c r="F16" s="32">
-        <f>IF(B16="","",IF(E16=TRUE,"✓ Paid",IF(D16&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D16-DAY(TODAY())&lt;=3,"Due in "&amp;(D16-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D16))))</f>
+        <f>IF(B16="","",IF(E16="Yes","Paid",IF(D16&lt;DAY(TODAY()),"Overdue",IF((D16-DAY(TODAY()))=0,"Due today",IF((D16-DAY(TODAY()))&lt;=3,"Due in "&amp;(D16-DAY(TODAY()))&amp;IF((D16-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D16&amp;IF(AND(D16&gt;=11,D16&lt;=13),"th",IF(MOD(D16,10)=1,"st",IF(MOD(D16,10)=2,"nd",IF(MOD(D16,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G16" s="1" t="n"/>
@@ -4387,7 +4410,7 @@
       <c r="D17" s="30" t="n"/>
       <c r="E17" s="31" t="n"/>
       <c r="F17" s="32">
-        <f>IF(B17="","",IF(E17=TRUE,"✓ Paid",IF(D17&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D17-DAY(TODAY())&lt;=3,"Due in "&amp;(D17-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D17))))</f>
+        <f>IF(B17="","",IF(E17="Yes","Paid",IF(D17&lt;DAY(TODAY()),"Overdue",IF((D17-DAY(TODAY()))=0,"Due today",IF((D17-DAY(TODAY()))&lt;=3,"Due in "&amp;(D17-DAY(TODAY()))&amp;IF((D17-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D17&amp;IF(AND(D17&gt;=11,D17&lt;=13),"th",IF(MOD(D17,10)=1,"st",IF(MOD(D17,10)=2,"nd",IF(MOD(D17,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G17" s="1" t="n"/>
@@ -4399,7 +4422,7 @@
       <c r="D18" s="30" t="n"/>
       <c r="E18" s="31" t="n"/>
       <c r="F18" s="32">
-        <f>IF(B18="","",IF(E18=TRUE,"✓ Paid",IF(D18&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D18-DAY(TODAY())&lt;=3,"Due in "&amp;(D18-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D18))))</f>
+        <f>IF(B18="","",IF(E18="Yes","Paid",IF(D18&lt;DAY(TODAY()),"Overdue",IF((D18-DAY(TODAY()))=0,"Due today",IF((D18-DAY(TODAY()))&lt;=3,"Due in "&amp;(D18-DAY(TODAY()))&amp;IF((D18-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D18&amp;IF(AND(D18&gt;=11,D18&lt;=13),"th",IF(MOD(D18,10)=1,"st",IF(MOD(D18,10)=2,"nd",IF(MOD(D18,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G18" s="1" t="n"/>
@@ -4411,7 +4434,7 @@
       <c r="D19" s="30" t="n"/>
       <c r="E19" s="31" t="n"/>
       <c r="F19" s="32">
-        <f>IF(B19="","",IF(E19=TRUE,"✓ Paid",IF(D19&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D19-DAY(TODAY())&lt;=3,"Due in "&amp;(D19-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D19))))</f>
+        <f>IF(B19="","",IF(E19="Yes","Paid",IF(D19&lt;DAY(TODAY()),"Overdue",IF((D19-DAY(TODAY()))=0,"Due today",IF((D19-DAY(TODAY()))&lt;=3,"Due in "&amp;(D19-DAY(TODAY()))&amp;IF((D19-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D19&amp;IF(AND(D19&gt;=11,D19&lt;=13),"th",IF(MOD(D19,10)=1,"st",IF(MOD(D19,10)=2,"nd",IF(MOD(D19,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G19" s="1" t="n"/>
@@ -4423,7 +4446,7 @@
       <c r="D20" s="30" t="n"/>
       <c r="E20" s="31" t="n"/>
       <c r="F20" s="32">
-        <f>IF(B20="","",IF(E20=TRUE,"✓ Paid",IF(D20&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D20-DAY(TODAY())&lt;=3,"Due in "&amp;(D20-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D20))))</f>
+        <f>IF(B20="","",IF(E20="Yes","Paid",IF(D20&lt;DAY(TODAY()),"Overdue",IF((D20-DAY(TODAY()))=0,"Due today",IF((D20-DAY(TODAY()))&lt;=3,"Due in "&amp;(D20-DAY(TODAY()))&amp;IF((D20-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D20&amp;IF(AND(D20&gt;=11,D20&lt;=13),"th",IF(MOD(D20,10)=1,"st",IF(MOD(D20,10)=2,"nd",IF(MOD(D20,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G20" s="1" t="n"/>
@@ -4435,7 +4458,7 @@
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="31" t="n"/>
       <c r="F21" s="32">
-        <f>IF(B21="","",IF(E21=TRUE,"✓ Paid",IF(D21&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D21-DAY(TODAY())&lt;=3,"Due in "&amp;(D21-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D21))))</f>
+        <f>IF(B21="","",IF(E21="Yes","Paid",IF(D21&lt;DAY(TODAY()),"Overdue",IF((D21-DAY(TODAY()))=0,"Due today",IF((D21-DAY(TODAY()))&lt;=3,"Due in "&amp;(D21-DAY(TODAY()))&amp;IF((D21-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D21&amp;IF(AND(D21&gt;=11,D21&lt;=13),"th",IF(MOD(D21,10)=1,"st",IF(MOD(D21,10)=2,"nd",IF(MOD(D21,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G21" s="1" t="n"/>
@@ -4447,7 +4470,7 @@
       <c r="D22" s="30" t="n"/>
       <c r="E22" s="31" t="n"/>
       <c r="F22" s="32">
-        <f>IF(B22="","",IF(E22=TRUE,"✓ Paid",IF(D22&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D22-DAY(TODAY())&lt;=3,"Due in "&amp;(D22-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D22))))</f>
+        <f>IF(B22="","",IF(E22="Yes","Paid",IF(D22&lt;DAY(TODAY()),"Overdue",IF((D22-DAY(TODAY()))=0,"Due today",IF((D22-DAY(TODAY()))&lt;=3,"Due in "&amp;(D22-DAY(TODAY()))&amp;IF((D22-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D22&amp;IF(AND(D22&gt;=11,D22&lt;=13),"th",IF(MOD(D22,10)=1,"st",IF(MOD(D22,10)=2,"nd",IF(MOD(D22,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G22" s="1" t="n"/>
@@ -4459,7 +4482,7 @@
       <c r="D23" s="30" t="n"/>
       <c r="E23" s="31" t="n"/>
       <c r="F23" s="32">
-        <f>IF(B23="","",IF(E23=TRUE,"✓ Paid",IF(D23&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D23-DAY(TODAY())&lt;=3,"Due in "&amp;(D23-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D23))))</f>
+        <f>IF(B23="","",IF(E23="Yes","Paid",IF(D23&lt;DAY(TODAY()),"Overdue",IF((D23-DAY(TODAY()))=0,"Due today",IF((D23-DAY(TODAY()))&lt;=3,"Due in "&amp;(D23-DAY(TODAY()))&amp;IF((D23-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D23&amp;IF(AND(D23&gt;=11,D23&lt;=13),"th",IF(MOD(D23,10)=1,"st",IF(MOD(D23,10)=2,"nd",IF(MOD(D23,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G23" s="1" t="n"/>
@@ -4471,7 +4494,7 @@
       <c r="D24" s="30" t="n"/>
       <c r="E24" s="31" t="n"/>
       <c r="F24" s="32">
-        <f>IF(B24="","",IF(E24=TRUE,"✓ Paid",IF(D24&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D24-DAY(TODAY())&lt;=3,"Due in "&amp;(D24-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D24))))</f>
+        <f>IF(B24="","",IF(E24="Yes","Paid",IF(D24&lt;DAY(TODAY()),"Overdue",IF((D24-DAY(TODAY()))=0,"Due today",IF((D24-DAY(TODAY()))&lt;=3,"Due in "&amp;(D24-DAY(TODAY()))&amp;IF((D24-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D24&amp;IF(AND(D24&gt;=11,D24&lt;=13),"th",IF(MOD(D24,10)=1,"st",IF(MOD(D24,10)=2,"nd",IF(MOD(D24,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G24" s="1" t="n"/>
@@ -4483,7 +4506,7 @@
       <c r="D25" s="30" t="n"/>
       <c r="E25" s="31" t="n"/>
       <c r="F25" s="32">
-        <f>IF(B25="","",IF(E25=TRUE,"✓ Paid",IF(D25&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D25-DAY(TODAY())&lt;=3,"Due in "&amp;(D25-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D25))))</f>
+        <f>IF(B25="","",IF(E25="Yes","Paid",IF(D25&lt;DAY(TODAY()),"Overdue",IF((D25-DAY(TODAY()))=0,"Due today",IF((D25-DAY(TODAY()))&lt;=3,"Due in "&amp;(D25-DAY(TODAY()))&amp;IF((D25-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D25&amp;IF(AND(D25&gt;=11,D25&lt;=13),"th",IF(MOD(D25,10)=1,"st",IF(MOD(D25,10)=2,"nd",IF(MOD(D25,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G25" s="1" t="n"/>
@@ -4495,7 +4518,7 @@
       <c r="D26" s="30" t="n"/>
       <c r="E26" s="31" t="n"/>
       <c r="F26" s="32">
-        <f>IF(B26="","",IF(E26=TRUE,"✓ Paid",IF(D26&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D26-DAY(TODAY())&lt;=3,"Due in "&amp;(D26-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D26))))</f>
+        <f>IF(B26="","",IF(E26="Yes","Paid",IF(D26&lt;DAY(TODAY()),"Overdue",IF((D26-DAY(TODAY()))=0,"Due today",IF((D26-DAY(TODAY()))&lt;=3,"Due in "&amp;(D26-DAY(TODAY()))&amp;IF((D26-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D26&amp;IF(AND(D26&gt;=11,D26&lt;=13),"th",IF(MOD(D26,10)=1,"st",IF(MOD(D26,10)=2,"nd",IF(MOD(D26,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G26" s="1" t="n"/>
@@ -4507,7 +4530,7 @@
       <c r="D27" s="30" t="n"/>
       <c r="E27" s="31" t="n"/>
       <c r="F27" s="32">
-        <f>IF(B27="","",IF(E27=TRUE,"✓ Paid",IF(D27&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D27-DAY(TODAY())&lt;=3,"Due in "&amp;(D27-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D27))))</f>
+        <f>IF(B27="","",IF(E27="Yes","Paid",IF(D27&lt;DAY(TODAY()),"Overdue",IF((D27-DAY(TODAY()))=0,"Due today",IF((D27-DAY(TODAY()))&lt;=3,"Due in "&amp;(D27-DAY(TODAY()))&amp;IF((D27-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D27&amp;IF(AND(D27&gt;=11,D27&lt;=13),"th",IF(MOD(D27,10)=1,"st",IF(MOD(D27,10)=2,"nd",IF(MOD(D27,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G27" s="1" t="n"/>
@@ -4519,7 +4542,7 @@
       <c r="D28" s="30" t="n"/>
       <c r="E28" s="31" t="n"/>
       <c r="F28" s="32">
-        <f>IF(B28="","",IF(E28=TRUE,"✓ Paid",IF(D28&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D28-DAY(TODAY())&lt;=3,"Due in "&amp;(D28-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D28))))</f>
+        <f>IF(B28="","",IF(E28="Yes","Paid",IF(D28&lt;DAY(TODAY()),"Overdue",IF((D28-DAY(TODAY()))=0,"Due today",IF((D28-DAY(TODAY()))&lt;=3,"Due in "&amp;(D28-DAY(TODAY()))&amp;IF((D28-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D28&amp;IF(AND(D28&gt;=11,D28&lt;=13),"th",IF(MOD(D28,10)=1,"st",IF(MOD(D28,10)=2,"nd",IF(MOD(D28,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G28" s="1" t="n"/>
@@ -4531,7 +4554,7 @@
       <c r="D29" s="30" t="n"/>
       <c r="E29" s="31" t="n"/>
       <c r="F29" s="32">
-        <f>IF(B29="","",IF(E29=TRUE,"✓ Paid",IF(D29&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D29-DAY(TODAY())&lt;=3,"Due in "&amp;(D29-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D29))))</f>
+        <f>IF(B29="","",IF(E29="Yes","Paid",IF(D29&lt;DAY(TODAY()),"Overdue",IF((D29-DAY(TODAY()))=0,"Due today",IF((D29-DAY(TODAY()))&lt;=3,"Due in "&amp;(D29-DAY(TODAY()))&amp;IF((D29-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D29&amp;IF(AND(D29&gt;=11,D29&lt;=13),"th",IF(MOD(D29,10)=1,"st",IF(MOD(D29,10)=2,"nd",IF(MOD(D29,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G29" s="1" t="n"/>
@@ -4543,7 +4566,7 @@
       <c r="D30" s="30" t="n"/>
       <c r="E30" s="31" t="n"/>
       <c r="F30" s="32">
-        <f>IF(B30="","",IF(E30=TRUE,"✓ Paid",IF(D30&lt;DAY(TODAY()),"⚠ OVERDUE",IF(D30-DAY(TODAY())&lt;=3,"Due in "&amp;(D30-DAY(TODAY()))&amp;" day(s)","Due on the "&amp;D30))))</f>
+        <f>IF(B30="","",IF(E30="Yes","Paid",IF(D30&lt;DAY(TODAY()),"Overdue",IF((D30-DAY(TODAY()))=0,"Due today",IF((D30-DAY(TODAY()))&lt;=3,"Due in "&amp;(D30-DAY(TODAY()))&amp;IF((D30-DAY(TODAY()))=1," day"," days"),"Due on the "&amp;D30&amp;IF(AND(D30&gt;=11,D30&lt;=13),"th",IF(MOD(D30,10)=1,"st",IF(MOD(D30,10)=2,"nd",IF(MOD(D30,10)=3,"rd","th")))))))))</f>
         <v/>
       </c>
       <c r="G30" s="1" t="n"/>
@@ -4992,18 +5015,18 @@
   </sheetData>
   <conditionalFormatting sqref="F6:F30">
     <cfRule type="expression" priority="1" dxfId="3">
-      <formula>LEFT($F6,1)="✓"</formula>
+      <formula>$F6="Paid"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>LEFT($F6,1)="⚠"</formula>
+      <formula>$F6="Overdue"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="4">
-      <formula>AND(LEFT($F6,6)="Due in",($D6-DAY(TODAY()))&lt;=3)</formula>
+      <formula>OR(LEFT($F6,6)="Due in",$F6="Due today")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="E6:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5056,7 +5079,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Want it? Park it here. If you still want it in 48 hours, go ahead.</t>
+          <t>Write down what you want to buy. If you still want it 48 hours later, go ahead.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -5122,7 +5145,7 @@
         <v>46290</v>
       </c>
       <c r="E6" s="34">
-        <f>IF(B6="","",IF(F6&lt;&gt;"",F6,IF(TODAY()-D6&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D6))&amp;" more day(s)")))</f>
+        <f>IF(B6="","",IF(F6&lt;&gt;"",F6,IF(TODAY()-D6&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D6))&amp;IF((2-(TODAY()-D6))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F6" s="31" t="inlineStr"/>
@@ -5146,7 +5169,7 @@
         <v>46292</v>
       </c>
       <c r="E7" s="34">
-        <f>IF(B7="","",IF(F7&lt;&gt;"",F7,IF(TODAY()-D7&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D7))&amp;" more day(s)")))</f>
+        <f>IF(B7="","",IF(F7&lt;&gt;"",F7,IF(TODAY()-D7&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D7))&amp;IF((2-(TODAY()-D7))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F7" s="31" t="inlineStr"/>
@@ -5166,7 +5189,7 @@
         <v>46287</v>
       </c>
       <c r="E8" s="34">
-        <f>IF(B8="","",IF(F8&lt;&gt;"",F8,IF(TODAY()-D8&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D8))&amp;" more day(s)")))</f>
+        <f>IF(B8="","",IF(F8&lt;&gt;"",F8,IF(TODAY()-D8&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D8))&amp;IF((2-(TODAY()-D8))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F8" s="31" t="inlineStr">
@@ -5190,7 +5213,7 @@
         <v>46284</v>
       </c>
       <c r="E9" s="34">
-        <f>IF(B9="","",IF(F9&lt;&gt;"",F9,IF(TODAY()-D9&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D9))&amp;" more day(s)")))</f>
+        <f>IF(B9="","",IF(F9&lt;&gt;"",F9,IF(TODAY()-D9&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D9))&amp;IF((2-(TODAY()-D9))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -5214,7 +5237,7 @@
         <v>46293</v>
       </c>
       <c r="E10" s="34">
-        <f>IF(B10="","",IF(F10&lt;&gt;"",F10,IF(TODAY()-D10&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D10))&amp;" more day(s)")))</f>
+        <f>IF(B10="","",IF(F10&lt;&gt;"",F10,IF(TODAY()-D10&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D10))&amp;IF((2-(TODAY()-D10))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F10" s="31" t="inlineStr"/>
@@ -5226,7 +5249,7 @@
       <c r="C11" s="28" t="n"/>
       <c r="D11" s="29" t="n"/>
       <c r="E11" s="34">
-        <f>IF(B11="","",IF(F11&lt;&gt;"",F11,IF(TODAY()-D11&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D11))&amp;" more day(s)")))</f>
+        <f>IF(B11="","",IF(F11&lt;&gt;"",F11,IF(TODAY()-D11&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D11))&amp;IF((2-(TODAY()-D11))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F11" s="31" t="n"/>
@@ -5238,7 +5261,7 @@
       <c r="C12" s="28" t="n"/>
       <c r="D12" s="29" t="n"/>
       <c r="E12" s="34">
-        <f>IF(B12="","",IF(F12&lt;&gt;"",F12,IF(TODAY()-D12&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D12))&amp;" more day(s)")))</f>
+        <f>IF(B12="","",IF(F12&lt;&gt;"",F12,IF(TODAY()-D12&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D12))&amp;IF((2-(TODAY()-D12))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F12" s="31" t="n"/>
@@ -5250,7 +5273,7 @@
       <c r="C13" s="28" t="n"/>
       <c r="D13" s="29" t="n"/>
       <c r="E13" s="34">
-        <f>IF(B13="","",IF(F13&lt;&gt;"",F13,IF(TODAY()-D13&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D13))&amp;" more day(s)")))</f>
+        <f>IF(B13="","",IF(F13&lt;&gt;"",F13,IF(TODAY()-D13&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D13))&amp;IF((2-(TODAY()-D13))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F13" s="31" t="n"/>
@@ -5262,7 +5285,7 @@
       <c r="C14" s="28" t="n"/>
       <c r="D14" s="29" t="n"/>
       <c r="E14" s="34">
-        <f>IF(B14="","",IF(F14&lt;&gt;"",F14,IF(TODAY()-D14&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D14))&amp;" more day(s)")))</f>
+        <f>IF(B14="","",IF(F14&lt;&gt;"",F14,IF(TODAY()-D14&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D14))&amp;IF((2-(TODAY()-D14))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F14" s="31" t="n"/>
@@ -5274,7 +5297,7 @@
       <c r="C15" s="28" t="n"/>
       <c r="D15" s="29" t="n"/>
       <c r="E15" s="34">
-        <f>IF(B15="","",IF(F15&lt;&gt;"",F15,IF(TODAY()-D15&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D15))&amp;" more day(s)")))</f>
+        <f>IF(B15="","",IF(F15&lt;&gt;"",F15,IF(TODAY()-D15&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D15))&amp;IF((2-(TODAY()-D15))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F15" s="31" t="n"/>
@@ -5286,7 +5309,7 @@
       <c r="C16" s="28" t="n"/>
       <c r="D16" s="29" t="n"/>
       <c r="E16" s="34">
-        <f>IF(B16="","",IF(F16&lt;&gt;"",F16,IF(TODAY()-D16&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D16))&amp;" more day(s)")))</f>
+        <f>IF(B16="","",IF(F16&lt;&gt;"",F16,IF(TODAY()-D16&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D16))&amp;IF((2-(TODAY()-D16))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F16" s="31" t="n"/>
@@ -5298,7 +5321,7 @@
       <c r="C17" s="28" t="n"/>
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="34">
-        <f>IF(B17="","",IF(F17&lt;&gt;"",F17,IF(TODAY()-D17&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D17))&amp;" more day(s)")))</f>
+        <f>IF(B17="","",IF(F17&lt;&gt;"",F17,IF(TODAY()-D17&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D17))&amp;IF((2-(TODAY()-D17))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F17" s="31" t="n"/>
@@ -5310,7 +5333,7 @@
       <c r="C18" s="28" t="n"/>
       <c r="D18" s="29" t="n"/>
       <c r="E18" s="34">
-        <f>IF(B18="","",IF(F18&lt;&gt;"",F18,IF(TODAY()-D18&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D18))&amp;" more day(s)")))</f>
+        <f>IF(B18="","",IF(F18&lt;&gt;"",F18,IF(TODAY()-D18&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D18))&amp;IF((2-(TODAY()-D18))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F18" s="31" t="n"/>
@@ -5322,7 +5345,7 @@
       <c r="C19" s="28" t="n"/>
       <c r="D19" s="29" t="n"/>
       <c r="E19" s="34">
-        <f>IF(B19="","",IF(F19&lt;&gt;"",F19,IF(TODAY()-D19&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D19))&amp;" more day(s)")))</f>
+        <f>IF(B19="","",IF(F19&lt;&gt;"",F19,IF(TODAY()-D19&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D19))&amp;IF((2-(TODAY()-D19))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F19" s="31" t="n"/>
@@ -5334,7 +5357,7 @@
       <c r="C20" s="28" t="n"/>
       <c r="D20" s="29" t="n"/>
       <c r="E20" s="34">
-        <f>IF(B20="","",IF(F20&lt;&gt;"",F20,IF(TODAY()-D20&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D20))&amp;" more day(s)")))</f>
+        <f>IF(B20="","",IF(F20&lt;&gt;"",F20,IF(TODAY()-D20&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D20))&amp;IF((2-(TODAY()-D20))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F20" s="31" t="n"/>
@@ -5346,7 +5369,7 @@
       <c r="C21" s="28" t="n"/>
       <c r="D21" s="29" t="n"/>
       <c r="E21" s="34">
-        <f>IF(B21="","",IF(F21&lt;&gt;"",F21,IF(TODAY()-D21&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D21))&amp;" more day(s)")))</f>
+        <f>IF(B21="","",IF(F21&lt;&gt;"",F21,IF(TODAY()-D21&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D21))&amp;IF((2-(TODAY()-D21))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F21" s="31" t="n"/>
@@ -5358,7 +5381,7 @@
       <c r="C22" s="28" t="n"/>
       <c r="D22" s="29" t="n"/>
       <c r="E22" s="34">
-        <f>IF(B22="","",IF(F22&lt;&gt;"",F22,IF(TODAY()-D22&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D22))&amp;" more day(s)")))</f>
+        <f>IF(B22="","",IF(F22&lt;&gt;"",F22,IF(TODAY()-D22&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D22))&amp;IF((2-(TODAY()-D22))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F22" s="31" t="n"/>
@@ -5370,7 +5393,7 @@
       <c r="C23" s="28" t="n"/>
       <c r="D23" s="29" t="n"/>
       <c r="E23" s="34">
-        <f>IF(B23="","",IF(F23&lt;&gt;"",F23,IF(TODAY()-D23&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D23))&amp;" more day(s)")))</f>
+        <f>IF(B23="","",IF(F23&lt;&gt;"",F23,IF(TODAY()-D23&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D23))&amp;IF((2-(TODAY()-D23))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F23" s="31" t="n"/>
@@ -5382,7 +5405,7 @@
       <c r="C24" s="28" t="n"/>
       <c r="D24" s="29" t="n"/>
       <c r="E24" s="34">
-        <f>IF(B24="","",IF(F24&lt;&gt;"",F24,IF(TODAY()-D24&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D24))&amp;" more day(s)")))</f>
+        <f>IF(B24="","",IF(F24&lt;&gt;"",F24,IF(TODAY()-D24&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D24))&amp;IF((2-(TODAY()-D24))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F24" s="31" t="n"/>
@@ -5394,7 +5417,7 @@
       <c r="C25" s="28" t="n"/>
       <c r="D25" s="29" t="n"/>
       <c r="E25" s="34">
-        <f>IF(B25="","",IF(F25&lt;&gt;"",F25,IF(TODAY()-D25&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D25))&amp;" more day(s)")))</f>
+        <f>IF(B25="","",IF(F25&lt;&gt;"",F25,IF(TODAY()-D25&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D25))&amp;IF((2-(TODAY()-D25))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F25" s="31" t="n"/>
@@ -5406,7 +5429,7 @@
       <c r="C26" s="28" t="n"/>
       <c r="D26" s="29" t="n"/>
       <c r="E26" s="34">
-        <f>IF(B26="","",IF(F26&lt;&gt;"",F26,IF(TODAY()-D26&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D26))&amp;" more day(s)")))</f>
+        <f>IF(B26="","",IF(F26&lt;&gt;"",F26,IF(TODAY()-D26&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D26))&amp;IF((2-(TODAY()-D26))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F26" s="31" t="n"/>
@@ -5418,7 +5441,7 @@
       <c r="C27" s="28" t="n"/>
       <c r="D27" s="29" t="n"/>
       <c r="E27" s="34">
-        <f>IF(B27="","",IF(F27&lt;&gt;"",F27,IF(TODAY()-D27&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D27))&amp;" more day(s)")))</f>
+        <f>IF(B27="","",IF(F27&lt;&gt;"",F27,IF(TODAY()-D27&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D27))&amp;IF((2-(TODAY()-D27))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F27" s="31" t="n"/>
@@ -5430,7 +5453,7 @@
       <c r="C28" s="28" t="n"/>
       <c r="D28" s="29" t="n"/>
       <c r="E28" s="34">
-        <f>IF(B28="","",IF(F28&lt;&gt;"",F28,IF(TODAY()-D28&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D28))&amp;" more day(s)")))</f>
+        <f>IF(B28="","",IF(F28&lt;&gt;"",F28,IF(TODAY()-D28&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D28))&amp;IF((2-(TODAY()-D28))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F28" s="31" t="n"/>
@@ -5442,7 +5465,7 @@
       <c r="C29" s="28" t="n"/>
       <c r="D29" s="29" t="n"/>
       <c r="E29" s="34">
-        <f>IF(B29="","",IF(F29&lt;&gt;"",F29,IF(TODAY()-D29&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D29))&amp;" more day(s)")))</f>
+        <f>IF(B29="","",IF(F29&lt;&gt;"",F29,IF(TODAY()-D29&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D29))&amp;IF((2-(TODAY()-D29))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F29" s="31" t="n"/>
@@ -5454,7 +5477,7 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
       <c r="E30" s="34">
-        <f>IF(B30="","",IF(F30&lt;&gt;"",F30,IF(TODAY()-D30&gt;=2,"✓ 48h passed: buy only if you still want it","⏳ Wait "&amp;(2-(TODAY()-D30))&amp;" more day(s)")))</f>
+        <f>IF(B30="","",IF(F30&lt;&gt;"",F30,IF(TODAY()-D30&gt;=2,"48 hours passed: buy it if you still want it","Wait "&amp;(2-(TODAY()-D30))&amp;IF((2-(TODAY()-D30))=1," more day"," more days"))))</f>
         <v/>
       </c>
       <c r="F30" s="31" t="n"/>
@@ -5904,10 +5927,10 @@
   </sheetData>
   <conditionalFormatting sqref="E6:E30">
     <cfRule type="expression" priority="1" dxfId="4">
-      <formula>LEFT($E6,1)="⏳"</formula>
+      <formula>LEFT($E6,4)="Wait"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="3">
-      <formula>LEFT($E6,1)="✓"</formula>
+      <formula>LEFT($E6,8)="48 hours"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="5">
       <formula>$E6="Skipped"</formula>

</xml_diff>